<commit_message>
align case timeline and entity names
</commit_message>
<xml_diff>
--- a/data/processed/case_relevant_bank_flows.xlsx
+++ b/data/processed/case_relevant_bank_flows.xlsx
@@ -546,7 +546,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>synthetic/wechat/张三/TenpayTrades.csv</t>
+          <t>synthetic/bank_flows/张三/TenpayTrades.csv</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -581,7 +581,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>微信转账</t>
+          <t>银行转账</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -591,29 +591,33 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2024-08-16 10:12:00</t>
+          <t>2008-08-16 10:12:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2024-08-16 10:12:00</t>
+          <t>2008-08-16 10:12:00</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>SYN-0</t>
+          <t>ORIG-2008</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>本轮合成数据将案情整体后移，微信交易时间即案情时间。</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>90000</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
+          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>90000</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -630,16 +634,21 @@
           <t>罗宇</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
           <t>借款</t>
         </is>
       </c>
-      <c r="U2" t="b">
-        <v>1</v>
-      </c>
-      <c r="V2" t="b">
-        <v>1</v>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -660,7 +669,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>synthetic/wechat/张三/TenpayTrades.csv</t>
+          <t>synthetic/bank_flows/张三/TenpayTrades.csv</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -695,7 +704,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>微信转账</t>
+          <t>银行转账</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -705,29 +714,33 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2024-08-16 10:18:00</t>
+          <t>2008-08-16 10:18:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2024-08-16 10:18:00</t>
+          <t>2008-08-16 10:18:00</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>SYN-0</t>
+          <t>ORIG-2008</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>本轮合成数据将案情整体后移，微信交易时间即案情时间。</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>80000</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
+          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>80000</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -744,16 +757,21 @@
           <t>陈三一</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
           <t>货款</t>
         </is>
       </c>
-      <c r="U3" t="b">
-        <v>1</v>
-      </c>
-      <c r="V3" t="b">
-        <v>1</v>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
@@ -774,7 +792,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>synthetic/wechat/张三/TenpayTrades.csv</t>
+          <t>synthetic/bank_flows/张三/TenpayTrades.csv</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -809,7 +827,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>微信转账</t>
+          <t>银行转账</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -819,29 +837,33 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2024-08-16 10:27:00</t>
+          <t>2008-08-16 10:27:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2024-08-16 10:27:00</t>
+          <t>2008-08-16 10:27:00</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>SYN-0</t>
+          <t>ORIG-2008</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>本轮合成数据将案情整体后移，微信交易时间即案情时间。</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
-        <v>100000</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
+          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -858,16 +880,21 @@
           <t>张夏天</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
           <t>往来款</t>
         </is>
       </c>
-      <c r="U4" t="b">
-        <v>1</v>
-      </c>
-      <c r="V4" t="b">
-        <v>1</v>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -888,7 +915,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>synthetic/wechat/罗宇/TenpayTrades.csv</t>
+          <t>synthetic/bank_flows/罗宇/TenpayTrades.csv</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -923,7 +950,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>微信转账</t>
+          <t>银行转账</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -933,29 +960,33 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2024-08-17 15:30:00</t>
+          <t>2008-08-17 15:30:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2024-08-17 15:30:00</t>
+          <t>2008-08-17 15:30:00</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SYN-0</t>
+          <t>ORIG-2008</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>本轮合成数据将案情整体后移，微信交易时间即案情时间。</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>90000</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
+          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>90000</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -972,16 +1003,21 @@
           <t>何晓初</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
           <t>还款</t>
         </is>
       </c>
-      <c r="U5" t="b">
-        <v>1</v>
-      </c>
-      <c r="V5" t="b">
-        <v>1</v>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -1002,7 +1038,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>synthetic/wechat/陈三一/TenpayTrades.csv</t>
+          <t>synthetic/bank_flows/陈三一/TenpayTrades.csv</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1037,7 +1073,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>微信转账</t>
+          <t>银行转账</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1047,29 +1083,33 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2024-08-18 09:48:00</t>
+          <t>2008-08-18 09:48:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2024-08-18 09:48:00</t>
+          <t>2008-08-18 09:48:00</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SYN-0</t>
+          <t>ORIG-2008</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>本轮合成数据将案情整体后移，微信交易时间即案情时间。</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
-        <v>80000</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
+          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>80000</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -1086,16 +1126,21 @@
           <t>何晓初控制账户</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
           <t>劳务费</t>
         </is>
       </c>
-      <c r="U6" t="b">
-        <v>1</v>
-      </c>
-      <c r="V6" t="b">
-        <v>1</v>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -1116,7 +1161,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>synthetic/wechat/张夏天/TenpayTrades.csv</t>
+          <t>synthetic/bank_flows/张夏天/TenpayTrades.csv</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1151,7 +1196,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>微信转账</t>
+          <t>银行转账</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1161,29 +1206,33 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2024-08-18 14:05:00</t>
+          <t>2008-08-18 14:05:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2024-08-18 14:05:00</t>
+          <t>2008-08-18 14:05:00</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SYN-0</t>
+          <t>ORIG-2008</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>本轮合成数据将案情整体后移，微信交易时间即案情时间。</t>
-        </is>
-      </c>
-      <c r="N7" t="n">
-        <v>100000</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
+          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -1200,16 +1249,21 @@
           <t>何晓初控制账户</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
           <t>投资款</t>
         </is>
       </c>
-      <c r="U7" t="b">
-        <v>1</v>
-      </c>
-      <c r="V7" t="b">
-        <v>1</v>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -1230,7 +1284,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>synthetic/wechat/张三/TenpayTrades.csv</t>
+          <t>synthetic/bank_flows/张三/TenpayTrades.csv</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1275,29 +1329,33 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2024-08-19 16:42:00</t>
+          <t>2008-08-19 16:42:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2024-08-19 16:42:00</t>
+          <t>2008-08-19 16:42:00</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SYN-0</t>
+          <t>ORIG-2008</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>本轮合成数据将案情整体后移，微信交易时间即案情时间。</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
-        <v>30000</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
+          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>30000</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -1314,16 +1372,21 @@
           <t>ATM</t>
         </is>
       </c>
+      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
           <t>现金备用</t>
         </is>
       </c>
-      <c r="U8" t="b">
-        <v>1</v>
-      </c>
-      <c r="V8" t="b">
-        <v>1</v>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -1344,7 +1407,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>synthetic/wechat/曾黎/TenpayTrades.csv</t>
+          <t>synthetic/bank_flows/曾黎/TenpayTrades.csv</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1389,29 +1452,33 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2024-08-21 10:08:00</t>
+          <t>2008-08-21 10:08:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2024-08-21 10:08:00</t>
+          <t>2008-08-21 10:08:00</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SYN-0</t>
+          <t>ORIG-2008</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>本轮合成数据将案情整体后移，微信交易时间即案情时间。</t>
-        </is>
-      </c>
-      <c r="N9" t="n">
-        <v>30000</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
+          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>30000</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
@@ -1428,16 +1495,21 @@
           <t>现金柜台</t>
         </is>
       </c>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
           <t>现金存入</t>
         </is>
       </c>
-      <c r="U9" t="b">
-        <v>1</v>
-      </c>
-      <c r="V9" t="b">
-        <v>1</v>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -1458,7 +1530,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>synthetic/wechat/李四/TenpayTrades.csv</t>
+          <t>synthetic/bank_flows/李四/TenpayTrades.csv</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1493,7 +1565,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>微信转账</t>
+          <t>银行转账</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1503,29 +1575,33 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2024-09-06 09:20:00</t>
+          <t>2008-09-06 09:20:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2024-09-06 09:20:00</t>
+          <t>2008-09-06 09:20:00</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SYN-0</t>
+          <t>ORIG-2008</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>本轮合成数据将案情整体后移，微信交易时间即案情时间。</t>
-        </is>
-      </c>
-      <c r="N10" t="n">
-        <v>50000</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
+          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>50000</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -1542,16 +1618,21 @@
           <t>江军</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
           <t>调解赔偿款</t>
         </is>
       </c>
-      <c r="U10" t="b">
-        <v>1</v>
-      </c>
-      <c r="V10" t="b">
-        <v>1</v>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
@@ -1572,7 +1653,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>synthetic/wechat/老刘/TenpayTrades.csv</t>
+          <t>synthetic/bank_flows/老刘/TenpayTrades.csv</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1607,7 +1688,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>微信转账</t>
+          <t>银行转账</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1617,29 +1698,33 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2024-09-06 09:31:00</t>
+          <t>2008-09-06 09:31:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2024-09-06 09:31:00</t>
+          <t>2008-09-06 09:31:00</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SYN-0</t>
+          <t>ORIG-2008</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>本轮合成数据将案情整体后移，微信交易时间即案情时间。</t>
-        </is>
-      </c>
-      <c r="N11" t="n">
-        <v>30000</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
+          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>30000</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -1656,16 +1741,21 @@
           <t>汪春蓉</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
           <t>调解赔偿款</t>
         </is>
       </c>
-      <c r="U11" t="b">
-        <v>1</v>
-      </c>
-      <c r="V11" t="b">
-        <v>1</v>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
@@ -1686,7 +1776,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>synthetic/wechat/老刘/TenpayTrades.csv</t>
+          <t>synthetic/bank_flows/老刘/TenpayTrades.csv</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1721,7 +1811,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>微信转账</t>
+          <t>银行转账</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1731,29 +1821,33 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2024-09-06 09:35:00</t>
+          <t>2008-09-06 09:35:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2024-09-06 09:35:00</t>
+          <t>2008-09-06 09:35:00</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SYN-0</t>
+          <t>ORIG-2008</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>本轮合成数据将案情整体后移，微信交易时间即案情时间。</t>
-        </is>
-      </c>
-      <c r="N12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0</v>
+          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>20000</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
@@ -1770,16 +1864,21 @@
           <t>赵志高</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
           <t>调解赔偿款</t>
         </is>
       </c>
-      <c r="U12" t="b">
-        <v>1</v>
-      </c>
-      <c r="V12" t="b">
-        <v>1</v>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
@@ -1800,7 +1899,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>synthetic/wechat/老刘/TenpayTrades.csv</t>
+          <t>synthetic/bank_flows/老刘/TenpayTrades.csv</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1835,7 +1934,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>微信转账</t>
+          <t>银行转账</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1845,29 +1944,33 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2024-09-06 09:39:00</t>
+          <t>2008-09-06 09:39:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2024-09-06 09:39:00</t>
+          <t>2008-09-06 09:39:00</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SYN-0</t>
+          <t>ORIG-2008</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>本轮合成数据将案情整体后移，微信交易时间即案情时间。</t>
-        </is>
-      </c>
-      <c r="N13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0</v>
+          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
@@ -1884,16 +1987,21 @@
           <t>易承桂</t>
         </is>
       </c>
+      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
           <t>调解赔偿款</t>
         </is>
       </c>
-      <c r="U13" t="b">
-        <v>1</v>
-      </c>
-      <c r="V13" t="b">
-        <v>1</v>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
restore future case timeline alignment
</commit_message>
<xml_diff>
--- a/data/processed/case_relevant_bank_flows.xlsx
+++ b/data/processed/case_relevant_bank_flows.xlsx
@@ -591,22 +591,22 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2008-08-16 10:12:00</t>
+          <t>2024-08-16 10:12:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2008-08-16 10:12:00</t>
+          <t>2024-08-16 10:12:00</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>ORIG-2008</t>
+          <t>FUTURE-16Y</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+          <t>本轮合成数据将原案整体后移16年，映射案情时间与银行流水/通话记录时间保持一致。</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2008-08-16 10:18:00</t>
+          <t>2024-08-16 10:18:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2008-08-16 10:18:00</t>
+          <t>2024-08-16 10:18:00</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>ORIG-2008</t>
+          <t>FUTURE-16Y</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+          <t>本轮合成数据将原案整体后移16年，映射案情时间与银行流水/通话记录时间保持一致。</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -837,22 +837,22 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2008-08-16 10:27:00</t>
+          <t>2024-08-16 10:27:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2008-08-16 10:27:00</t>
+          <t>2024-08-16 10:27:00</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>ORIG-2008</t>
+          <t>FUTURE-16Y</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+          <t>本轮合成数据将原案整体后移16年，映射案情时间与银行流水/通话记录时间保持一致。</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -960,22 +960,22 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2008-08-17 15:30:00</t>
+          <t>2024-08-17 15:30:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2008-08-17 15:30:00</t>
+          <t>2024-08-17 15:30:00</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>ORIG-2008</t>
+          <t>FUTURE-16Y</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+          <t>本轮合成数据将原案整体后移16年，映射案情时间与银行流水/通话记录时间保持一致。</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1083,22 +1083,22 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2008-08-18 09:48:00</t>
+          <t>2024-08-18 09:48:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2008-08-18 09:48:00</t>
+          <t>2024-08-18 09:48:00</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>ORIG-2008</t>
+          <t>FUTURE-16Y</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+          <t>本轮合成数据将原案整体后移16年，映射案情时间与银行流水/通话记录时间保持一致。</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1206,22 +1206,22 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2008-08-18 14:05:00</t>
+          <t>2024-08-18 14:05:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2008-08-18 14:05:00</t>
+          <t>2024-08-18 14:05:00</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>ORIG-2008</t>
+          <t>FUTURE-16Y</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+          <t>本轮合成数据将原案整体后移16年，映射案情时间与银行流水/通话记录时间保持一致。</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1329,22 +1329,22 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2008-08-19 16:42:00</t>
+          <t>2024-08-19 16:42:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2008-08-19 16:42:00</t>
+          <t>2024-08-19 16:42:00</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>ORIG-2008</t>
+          <t>FUTURE-16Y</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+          <t>本轮合成数据将原案整体后移16年，映射案情时间与银行流水/通话记录时间保持一致。</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1452,22 +1452,22 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2008-08-21 10:08:00</t>
+          <t>2024-08-21 10:08:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2008-08-21 10:08:00</t>
+          <t>2024-08-21 10:08:00</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>ORIG-2008</t>
+          <t>FUTURE-16Y</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+          <t>本轮合成数据将原案整体后移16年，映射案情时间与银行流水/通话记录时间保持一致。</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1575,22 +1575,22 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2008-09-06 09:20:00</t>
+          <t>2024-09-06 09:20:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2008-09-06 09:20:00</t>
+          <t>2024-09-06 09:20:00</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>ORIG-2008</t>
+          <t>FUTURE-16Y</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+          <t>本轮合成数据将原案整体后移16年，映射案情时间与银行流水/通话记录时间保持一致。</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1698,22 +1698,22 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2008-09-06 09:31:00</t>
+          <t>2024-09-06 09:31:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2008-09-06 09:31:00</t>
+          <t>2024-09-06 09:31:00</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>ORIG-2008</t>
+          <t>FUTURE-16Y</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+          <t>本轮合成数据将原案整体后移16年，映射案情时间与银行流水/通话记录时间保持一致。</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1821,22 +1821,22 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2008-09-06 09:35:00</t>
+          <t>2024-09-06 09:35:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2008-09-06 09:35:00</t>
+          <t>2024-09-06 09:35:00</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>ORIG-2008</t>
+          <t>FUTURE-16Y</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+          <t>本轮合成数据将原案整体后移16年，映射案情时间与银行流水/通话记录时间保持一致。</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1944,22 +1944,22 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2008-09-06 09:39:00</t>
+          <t>2024-09-06 09:39:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2008-09-06 09:39:00</t>
+          <t>2024-09-06 09:39:00</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>ORIG-2008</t>
+          <t>FUTURE-16Y</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>合成测试数据已与原始案情时间线对齐：原2023-2024样本整体映射回2007-2008案情节点；交易/通话时间以映射案情时间为准。</t>
+          <t>本轮合成数据将原案整体后移16年，映射案情时间与银行流水/通话记录时间保持一致。</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">

</xml_diff>